<commit_message>
add concat_text and refactor concat to concat_columns
</commit_message>
<xml_diff>
--- a/catalogo_operaciones.xlsx
+++ b/catalogo_operaciones.xlsx
@@ -8,7 +8,9 @@
   <sheets>
     <sheet name="Operaciones" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Operaciones'!$A$1:$D$100</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -175,7 +177,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="OperationsCatalog" displayName="OperationsCatalog" ref="A1:D99" headerRowCount="1" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="OperationsCatalog" displayName="OperationsCatalog" ref="A1:D100" headerRowCount="1" totalsRowShown="0">
   <autoFilter ref="A1:D99"/>
   <tableColumns count="4">
     <tableColumn id="1" name="Nombre exacto de la función"/>
@@ -476,7 +478,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D99"/>
+  <dimension ref="A1:D100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32.005" bestFit="1" customWidth="1" style="4" min="1" max="1"/>
@@ -1884,7 +1886,7 @@
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, delimiter: str, index: int | None = None, create_new_column: bool = False, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, delimiter: str, index: int | None = None, create_new_column: bool = True, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
@@ -1896,7 +1898,7 @@
     <row r="65" ht="38" customFormat="1" customHeight="1" s="1">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>concat</t>
+          <t>concat_column</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
@@ -1906,12 +1908,12 @@
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, columns: list[str], separator: str = '', create_new_column: bool = False, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, columns: list[str], separator: str = '', create_new_column: bool = True, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>Concatena dos o más columnas de texto usando el separador indicado.</t>
+          <t>Concatena dos o más columnas de texto y crea por defecto una columna nueva; los valores nulos de las columnas de entrada se propagan al resultado.</t>
         </is>
       </c>
     </row>
@@ -1928,7 +1930,7 @@
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, search_text: str, create_new_column: bool = False, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, search_text: str, create_new_column: bool = True, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
@@ -1950,7 +1952,7 @@
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, search_text: str, create_new_column: bool = False, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, search_text: str, create_new_column: bool = True, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr">
@@ -1972,7 +1974,7 @@
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, search_text: str, create_new_column: bool = False, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, search_text: str, create_new_column: bool = True, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D68" s="3" t="inlineStr">
@@ -2038,7 +2040,7 @@
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, create_new_column: bool = False, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, create_new_column: bool = True, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
@@ -2663,7 +2665,30 @@
         </is>
       </c>
     </row>
+    <row r="100" ht="42" customHeight="1">
+      <c r="A100" s="3" t="inlineStr">
+        <is>
+          <t>concat_text</t>
+        </is>
+      </c>
+      <c r="B100" s="3" t="inlineStr">
+        <is>
+          <t>TextProcessor</t>
+        </is>
+      </c>
+      <c r="C100" s="3" t="inlineStr">
+        <is>
+          <t>df: pd.DataFrame, column_name: str, value: str, create_new_column: bool = False, new_column_name: str | None = None</t>
+        </is>
+      </c>
+      <c r="D100" s="3" t="inlineStr">
+        <is>
+          <t>Concatena un texto literal al contenido de la columna y reemplaza por defecto su valor; puede crear una columna nueva si se solicita.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="A1:D100"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>

<commit_message>
Move sort to rows
</commit_message>
<xml_diff>
--- a/catalogo_operaciones.xlsx
+++ b/catalogo_operaciones.xlsx
@@ -9,7 +9,7 @@
     <sheet name="Operaciones" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Operaciones'!$A$1:$D$100</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Operaciones'!$A$1:$D$102</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -177,7 +177,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="OperationsCatalog" displayName="OperationsCatalog" ref="A1:D100" headerRowCount="1" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="OperationsCatalog" displayName="OperationsCatalog" ref="A1:D102" headerRowCount="1" totalsRowShown="0">
   <autoFilter ref="A1:D99"/>
   <tableColumns count="4">
     <tableColumn id="1" name="Nombre exacto de la función"/>
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D100"/>
+  <dimension ref="A1:D102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32.005" bestFit="1" customWidth="1" style="4" min="1" max="1"/>
@@ -1455,10 +1455,10 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="38" customFormat="1" customHeight="1" s="1">
+    <row r="45" ht="42" customFormat="1" customHeight="1" s="1">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>add_column</t>
+          <t>left_join</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -1468,19 +1468,19 @@
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column_name: str, value: object = None</t>
+          <t>left: pd.DataFrame, right: pd.DataFrame, *, how: str = 'left', left_on: str | list[str] | None = None, right_on: str | list[str] | None = None, suffixes: Sequence[str] = ('_x', '_y')</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>Agrega una columna nueva con el valor constante indicado.</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="38" customFormat="1" customHeight="1" s="1">
+          <t>Realiza una unión left entre dos DataFrames; conserva todas las filas del DataFrame izquierdo y las coincidencias del derecho.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="42" customFormat="1" customHeight="1" s="1">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>sort</t>
+          <t>right_join</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
@@ -1490,19 +1490,19 @@
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, direction: str = 'asc'</t>
+          <t>left: pd.DataFrame, right: pd.DataFrame, *, how: str = 'right', left_on: str | list[str] | None = None, right_on: str | list[str] | None = None, suffixes: Sequence[str] = ('_x', '_y')</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>Ordena las filas por una columna en orden ascendente o descendente.</t>
+          <t>Realiza una unión right entre dos DataFrames; conserva todas las filas del DataFrame derecho y las coincidencias del izquierdo.</t>
         </is>
       </c>
     </row>
     <row r="47" ht="38" customFormat="1" customHeight="1" s="1">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>drop-column</t>
+          <t>add_column</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -1512,41 +1512,41 @@
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str | Sequence[str] | None = None, *, columns: Sequence[str] | None = None</t>
+          <t>df: pd.DataFrame, column_name: str, value: object = None</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>Elimina una o varias columnas del DataFrame.</t>
+          <t>Agrega una columna nueva con el valor constante indicado.</t>
         </is>
       </c>
     </row>
     <row r="48" ht="38" customFormat="1" customHeight="1" s="1">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>drop_column</t>
+          <t>sort</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>StructuralProcessor</t>
+          <t>RowProcessor</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str | Sequence[str] | None = None, *, columns: Sequence[str] | None = None</t>
+          <t>df: pd.DataFrame, column: str, direction: str = 'asc'</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>Elimina una o varias columnas del DataFrame.</t>
+          <t>Ordena las filas por una columna en orden ascendente o descendente.</t>
         </is>
       </c>
     </row>
     <row r="49" ht="38" customFormat="1" customHeight="1" s="1">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>rename-column</t>
+          <t>drop-column</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -1556,19 +1556,19 @@
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, new_name: str</t>
+          <t>df: pd.DataFrame, column: str | Sequence[str] | None = None, *, columns: Sequence[str] | None = None</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>Renombra una columna existente.</t>
+          <t>Elimina una o varias columnas del DataFrame.</t>
         </is>
       </c>
     </row>
     <row r="50" ht="38" customFormat="1" customHeight="1" s="1">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>rename_column</t>
+          <t>drop_column</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
@@ -1578,19 +1578,19 @@
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, new_name: str</t>
+          <t>df: pd.DataFrame, column: str | Sequence[str] | None = None, *, columns: Sequence[str] | None = None</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>Renombra una columna existente.</t>
+          <t>Elimina una o varias columnas del DataFrame.</t>
         </is>
       </c>
     </row>
     <row r="51" ht="38" customFormat="1" customHeight="1" s="1">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>change-data-type</t>
+          <t>rename-column</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
@@ -1600,19 +1600,19 @@
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, new_type: str | None = None, *, target_type: str | None = None, create_new_column: bool | None = None, new_column: bool = False, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, new_name: str</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>Convierte una columna al tipo de dato especificado.</t>
+          <t>Renombra una columna existente.</t>
         </is>
       </c>
     </row>
     <row r="52" ht="38" customFormat="1" customHeight="1" s="1">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>change_data_type</t>
+          <t>rename_column</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
@@ -1622,19 +1622,19 @@
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, new_type: str | None = None, *, target_type: str | None = None, create_new_column: bool | None = None, new_column: bool = False, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, new_name: str</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>Convierte una columna al tipo de dato especificado.</t>
+          <t>Renombra una columna existente.</t>
         </is>
       </c>
     </row>
     <row r="53" ht="38" customFormat="1" customHeight="1" s="1">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>aggregate</t>
+          <t>change-data-type</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
@@ -1644,19 +1644,19 @@
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, group_by: list[str], aggregations: dict[str, str | list[str]]</t>
+          <t>df: pd.DataFrame, column: str, new_type: str | None = None, *, target_type: str | None = None, create_new_column: bool | None = None, new_column: bool = False, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>Agrupa filas y calcula las agregaciones solicitadas; conserva claves de agrupación nulas.</t>
+          <t>Convierte una columna al tipo de dato especificado.</t>
         </is>
       </c>
     </row>
     <row r="54" ht="38" customFormat="1" customHeight="1" s="1">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>pivot</t>
+          <t>change_data_type</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
@@ -1666,63 +1666,63 @@
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, pivot_type: str, index_cols: list[str], target_col: str, values_col: str</t>
+          <t>df: pd.DataFrame, column: str, new_type: str | None = None, *, target_type: str | None = None, create_new_column: bool | None = None, new_column: bool = False, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>Reestructura datos entre formato columnas-a-filas y filas-a-columnas.</t>
+          <t>Convierte una columna al tipo de dato especificado.</t>
         </is>
       </c>
     </row>
     <row r="55" ht="38" customFormat="1" customHeight="1" s="1">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>uppercase</t>
+          <t>aggregate</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>TextProcessor</t>
+          <t>StructuralProcessor</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, new_column: bool = False, new_column_name: str | None = None, *, create_new_column: bool | None = None</t>
+          <t>df: pd.DataFrame, group_by: list[str], aggregations: dict[str, str | list[str]]</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>Convierte el texto de una columna a mayúsculas.</t>
+          <t>Agrupa filas y calcula las agregaciones solicitadas; conserva claves de agrupación nulas.</t>
         </is>
       </c>
     </row>
     <row r="56" ht="38" customFormat="1" customHeight="1" s="1">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>upper</t>
+          <t>pivot</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>TextProcessor</t>
+          <t>StructuralProcessor</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, new_column: bool = False, new_column_name: str | None = None, *, create_new_column: bool | None = None</t>
+          <t>df: pd.DataFrame, pivot_type: str, index_cols: list[str], target_col: str, values_col: str</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>Alias de uppercase: convierte el texto de una columna a mayúsculas.</t>
+          <t>Reestructura datos entre formato columnas-a-filas y filas-a-columnas.</t>
         </is>
       </c>
     </row>
     <row r="57" ht="38" customFormat="1" customHeight="1" s="1">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>lowercase</t>
+          <t>uppercase</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
@@ -1737,14 +1737,14 @@
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>Convierte el texto de una columna a minúsculas.</t>
+          <t>Convierte el texto de una columna a mayúsculas.</t>
         </is>
       </c>
     </row>
     <row r="58" ht="38" customFormat="1" customHeight="1" s="1">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>lower</t>
+          <t>upper</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
@@ -1759,14 +1759,14 @@
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>Alias de lowercase: convierte el texto de una columna a minúsculas.</t>
+          <t>Alias de uppercase: convierte el texto de una columna a mayúsculas.</t>
         </is>
       </c>
     </row>
     <row r="59" ht="38" customFormat="1" customHeight="1" s="1">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>trim</t>
+          <t>lowercase</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
@@ -1776,19 +1776,19 @@
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, create_new_column: bool = False, new_column_name: str | None = None, *, side: str = 'both'</t>
+          <t>df: pd.DataFrame, column: str, new_column: bool = False, new_column_name: str | None = None, *, create_new_column: bool | None = None</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>Elimina espacios en blanco al inicio, al final o en ambos lados del texto.</t>
+          <t>Convierte el texto de una columna a minúsculas.</t>
         </is>
       </c>
     </row>
     <row r="60" ht="38" customFormat="1" customHeight="1" s="1">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>ltrim</t>
+          <t>lower</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
@@ -1798,19 +1798,19 @@
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, create_new_column: bool = False, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, new_column: bool = False, new_column_name: str | None = None, *, create_new_column: bool | None = None</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>Elimina espacios en blanco al inicio del texto.</t>
+          <t>Alias de lowercase: convierte el texto de una columna a minúsculas.</t>
         </is>
       </c>
     </row>
     <row r="61" ht="38" customFormat="1" customHeight="1" s="1">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>rtrim</t>
+          <t>trim</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
@@ -1820,19 +1820,19 @@
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, create_new_column: bool = False, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, create_new_column: bool = False, new_column_name: str | None = None, *, side: str = 'both'</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>Elimina espacios en blanco al final del texto.</t>
+          <t>Elimina espacios en blanco al inicio, al final o en ambos lados del texto.</t>
         </is>
       </c>
     </row>
     <row r="62" ht="38" customFormat="1" customHeight="1" s="1">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>substring</t>
+          <t>ltrim</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
@@ -1842,19 +1842,19 @@
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, start: int, length: int, create_new_column: bool = False, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, create_new_column: bool = False, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>Extrae una subcadena usando posiciones de índice desde cero.</t>
+          <t>Elimina espacios en blanco al inicio del texto.</t>
         </is>
       </c>
     </row>
     <row r="63" ht="38" customFormat="1" customHeight="1" s="1">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>replace</t>
+          <t>rtrim</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
@@ -1864,19 +1864,19 @@
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, old_text: str, new_text: str, create_new_column: bool = False, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, create_new_column: bool = False, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>Reemplaza todas las apariciones literales de un texto por otro.</t>
+          <t>Elimina espacios en blanco al final del texto.</t>
         </is>
       </c>
     </row>
     <row r="64" ht="38" customFormat="1" customHeight="1" s="1">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>split</t>
+          <t>substring</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
@@ -1886,19 +1886,19 @@
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, delimiter: str, index: int | None = None, create_new_column: bool = True, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, start: int, length: int, create_new_column: bool = False, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>Divide texto por un delimitador; extrae un índice o expande las partes en columnas nuevas.</t>
+          <t>Extrae una subcadena usando posiciones de índice desde cero.</t>
         </is>
       </c>
     </row>
     <row r="65" ht="38" customFormat="1" customHeight="1" s="1">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>concat_column</t>
+          <t>replace</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
@@ -1908,19 +1908,19 @@
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, columns: list[str], separator: str = '', create_new_column: bool = True, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, old_text: str, new_text: str, create_new_column: bool = False, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>Concatena dos o más columnas de texto y crea por defecto una columna nueva; los valores nulos de las columnas de entrada se propagan al resultado.</t>
+          <t>Reemplaza todas las apariciones literales de un texto por otro.</t>
         </is>
       </c>
     </row>
     <row r="66" ht="42" customFormat="1" customHeight="1" s="1">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>contains</t>
+          <t>split</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
@@ -1930,19 +1930,19 @@
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, search_text: str, create_new_column: bool = True, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, delimiter: str, index: int | None = None, create_new_column: bool = True, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>Devuelve True si el texto de cada celda contiene literalmente search_text; en caso contrario False. Los nulos producen False.</t>
+          <t>Divide texto por un delimitador; extrae un índice o expande las partes en columnas nuevas.</t>
         </is>
       </c>
     </row>
     <row r="67" ht="42" customFormat="1" customHeight="1" s="1">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>starts_with</t>
+          <t>concat_column</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
@@ -1952,19 +1952,19 @@
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, search_text: str, create_new_column: bool = True, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, columns: list[str], separator: str = '', create_new_column: bool = True, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>Devuelve True si el texto de cada celda comienza literalmente con search_text; en caso contrario False. Los nulos producen False.</t>
+          <t>Concatena dos o más columnas de texto y crea por defecto una columna nueva; los valores nulos de las columnas de entrada se propagan al resultado.</t>
         </is>
       </c>
     </row>
     <row r="68" ht="42" customFormat="1" customHeight="1" s="1">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>ends_with</t>
+          <t>contains</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
@@ -1979,14 +1979,14 @@
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>Devuelve True si el texto de cada celda termina literalmente con search_text; en caso contrario False. Los nulos producen False.</t>
+          <t>Devuelve True si el texto de cada celda contiene literalmente search_text; en caso contrario False. Los nulos producen False.</t>
         </is>
       </c>
     </row>
     <row r="69" ht="42" customFormat="1" customHeight="1" s="1">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>transform_left</t>
+          <t>starts_with</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
@@ -1996,19 +1996,19 @@
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, limit: int, create_new_column: bool = False, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, search_text: str, create_new_column: bool = True, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>Conserva como máximo los primeros limit caracteres de cada valor.</t>
+          <t>Devuelve True si el texto de cada celda comienza literalmente con search_text; en caso contrario False. Los nulos producen False.</t>
         </is>
       </c>
     </row>
     <row r="70" ht="42" customFormat="1" customHeight="1" s="1">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>transform_right</t>
+          <t>ends_with</t>
         </is>
       </c>
       <c r="B70" s="3" t="inlineStr">
@@ -2018,19 +2018,19 @@
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, limit: int, create_new_column: bool = False, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, search_text: str, create_new_column: bool = True, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>Conserva como máximo los últimos limit caracteres de cada valor.</t>
+          <t>Devuelve True si el texto de cada celda termina literalmente con search_text; en caso contrario False. Los nulos producen False.</t>
         </is>
       </c>
     </row>
     <row r="71" ht="42" customFormat="1" customHeight="1" s="1">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>length</t>
+          <t>transform_left</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
@@ -2040,19 +2040,19 @@
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, create_new_column: bool = True, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, limit: int, create_new_column: bool = False, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>Calcula la longitud en caracteres de cada celda; los valores nulos se mantienen nulos.</t>
+          <t>Conserva como máximo los primeros limit caracteres de cada valor.</t>
         </is>
       </c>
     </row>
     <row r="72" ht="42" customFormat="1" customHeight="1" s="1">
       <c r="A72" s="3" t="inlineStr">
         <is>
-          <t>proper</t>
+          <t>transform_right</t>
         </is>
       </c>
       <c r="B72" s="3" t="inlineStr">
@@ -2062,19 +2062,19 @@
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, new_column: bool = False, new_column_name: str | None = None, *, create_new_column: bool | None = None</t>
+          <t>df: pd.DataFrame, column: str, limit: int, create_new_column: bool = False, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>Convierte la primera letra de cada palabra a mayúscula y el resto a minúscula; puede reemplazar la columna o crear una nueva.</t>
+          <t>Conserva como máximo los últimos limit caracteres de cada valor.</t>
         </is>
       </c>
     </row>
     <row r="73" ht="42" customFormat="1" customHeight="1" s="1">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>propper</t>
+          <t>length</t>
         </is>
       </c>
       <c r="B73" s="3" t="inlineStr">
@@ -2084,63 +2084,63 @@
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, new_column: bool = False, new_column_name: str | None = None, *, create_new_column: bool | None = None</t>
+          <t>df: pd.DataFrame, column: str, create_new_column: bool = True, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>Alias de proper: convierte la primera letra de cada palabra a mayúscula y el resto a minúscula; puede reemplazar la columna o crear una nueva.</t>
+          <t>Calcula la longitud en caracteres de cada celda; los valores nulos se mantienen nulos.</t>
         </is>
       </c>
     </row>
     <row r="74" ht="42" customFormat="1" customHeight="1" s="1">
       <c r="A74" s="3" t="inlineStr">
         <is>
-          <t>date_parse</t>
+          <t>proper</t>
         </is>
       </c>
       <c r="B74" s="3" t="inlineStr">
         <is>
-          <t>DateTimeProcessor</t>
+          <t>TextProcessor</t>
         </is>
       </c>
       <c r="C74" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, date_format: str, replace: bool = True, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, new_column: bool = False, new_column_name: str | None = None, *, create_new_column: bool | None = None</t>
         </is>
       </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
-          <t>Convierte usando el formato indicado; los valores inválidos se convierten a NaT. Puede reemplazar o crear columna.</t>
+          <t>Convierte la primera letra de cada palabra a mayúscula y el resto a minúscula; puede reemplazar la columna o crear una nueva.</t>
         </is>
       </c>
     </row>
     <row r="75" ht="42" customFormat="1" customHeight="1" s="1">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>dateparse</t>
+          <t>propper</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>DateTimeProcessor</t>
+          <t>TextProcessor</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, date_format: str, replace: bool = True, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, new_column: bool = False, new_column_name: str | None = None, *, create_new_column: bool | None = None</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>Alias normalizado de date_parse; los valores inválidos se convierten a NaT.</t>
+          <t>Alias de proper: convierte la primera letra de cada palabra a mayúscula y el resto a minúscula; puede reemplazar la columna o crear una nueva.</t>
         </is>
       </c>
     </row>
     <row r="76" ht="42" customFormat="1" customHeight="1" s="1">
       <c r="A76" s="3" t="inlineStr">
         <is>
-          <t>date_trunc</t>
+          <t>date_parse</t>
         </is>
       </c>
       <c r="B76" s="3" t="inlineStr">
@@ -2150,19 +2150,19 @@
       </c>
       <c r="C76" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, part: str, replace: bool = True, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, date_format: str, replace: bool = True, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t>Trunca la fecha al inicio de año, trimestre, mes, semana (lunes), día, hora, minuto o segundo.</t>
+          <t>Convierte usando el formato indicado; los valores inválidos se convierten a NaT. Puede reemplazar o crear columna.</t>
         </is>
       </c>
     </row>
     <row r="77" ht="42" customFormat="1" customHeight="1" s="1">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>datetrunc</t>
+          <t>dateparse</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
@@ -2172,19 +2172,19 @@
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, part: str, replace: bool = True, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, date_format: str, replace: bool = True, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t>Alias normalizado de date_trunc.</t>
+          <t>Alias normalizado de date_parse; los valores inválidos se convierten a NaT.</t>
         </is>
       </c>
     </row>
     <row r="78" ht="42" customFormat="1" customHeight="1" s="1">
       <c r="A78" s="3" t="inlineStr">
         <is>
-          <t>day</t>
+          <t>date_trunc</t>
         </is>
       </c>
       <c r="B78" s="3" t="inlineStr">
@@ -2194,19 +2194,19 @@
       </c>
       <c r="C78" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, replace: bool = True, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, part: str, replace: bool = True, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D78" s="3" t="inlineStr">
         <is>
-          <t>Extrae el día del mes como entero.</t>
+          <t>Trunca la fecha al inicio de año, trimestre, mes, semana (lunes), día, hora, minuto o segundo.</t>
         </is>
       </c>
     </row>
     <row r="79" ht="42" customFormat="1" customHeight="1" s="1">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>iso_quarter</t>
+          <t>datetrunc</t>
         </is>
       </c>
       <c r="B79" s="3" t="inlineStr">
@@ -2216,19 +2216,19 @@
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, replace: bool = True, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, part: str, replace: bool = True, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
-          <t>Calcula el trimestre basado en semanas ISO; la semana 53 pertenece al trimestre 4.</t>
+          <t>Alias normalizado de date_trunc.</t>
         </is>
       </c>
     </row>
     <row r="80" ht="42" customFormat="1" customHeight="1" s="1">
       <c r="A80" s="3" t="inlineStr">
         <is>
-          <t>isoquarter</t>
+          <t>day</t>
         </is>
       </c>
       <c r="B80" s="3" t="inlineStr">
@@ -2243,14 +2243,14 @@
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t>Alias normalizado de iso_quarter.</t>
+          <t>Extrae el día del mes como entero.</t>
         </is>
       </c>
     </row>
     <row r="81" ht="42" customFormat="1" customHeight="1" s="1">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>iso_week</t>
+          <t>iso_quarter</t>
         </is>
       </c>
       <c r="B81" s="3" t="inlineStr">
@@ -2265,14 +2265,14 @@
       </c>
       <c r="D81" s="3" t="inlineStr">
         <is>
-          <t>Extrae el número de semana ISO 8601 como entero.</t>
+          <t>Calcula el trimestre basado en semanas ISO; la semana 53 pertenece al trimestre 4.</t>
         </is>
       </c>
     </row>
     <row r="82" ht="42" customFormat="1" customHeight="1" s="1">
       <c r="A82" s="3" t="inlineStr">
         <is>
-          <t>isoweek</t>
+          <t>isoquarter</t>
         </is>
       </c>
       <c r="B82" s="3" t="inlineStr">
@@ -2287,14 +2287,14 @@
       </c>
       <c r="D82" s="3" t="inlineStr">
         <is>
-          <t>Alias normalizado de iso_week.</t>
+          <t>Alias normalizado de iso_quarter.</t>
         </is>
       </c>
     </row>
     <row r="83" ht="42" customFormat="1" customHeight="1" s="1">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>iso_week_day</t>
+          <t>iso_week</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
@@ -2309,14 +2309,14 @@
       </c>
       <c r="D83" s="3" t="inlineStr">
         <is>
-          <t>Extrae el día de la semana ISO 8601: lunes=1 hasta domingo=7.</t>
+          <t>Extrae el número de semana ISO 8601 como entero.</t>
         </is>
       </c>
     </row>
     <row r="84" ht="42" customFormat="1" customHeight="1" s="1">
       <c r="A84" s="3" t="inlineStr">
         <is>
-          <t>isoweekday</t>
+          <t>isoweek</t>
         </is>
       </c>
       <c r="B84" s="3" t="inlineStr">
@@ -2331,14 +2331,14 @@
       </c>
       <c r="D84" s="3" t="inlineStr">
         <is>
-          <t>Alias normalizado de iso_week_day.</t>
+          <t>Alias normalizado de iso_week.</t>
         </is>
       </c>
     </row>
     <row r="85" ht="42" customFormat="1" customHeight="1" s="1">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>iso_year</t>
+          <t>iso_week_day</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
@@ -2353,14 +2353,14 @@
       </c>
       <c r="D85" s="3" t="inlineStr">
         <is>
-          <t>Extrae el año ISO 8601, que puede diferir del año calendario.</t>
+          <t>Extrae el día de la semana ISO 8601: lunes=1 hasta domingo=7.</t>
         </is>
       </c>
     </row>
     <row r="86" ht="42" customFormat="1" customHeight="1" s="1">
       <c r="A86" s="3" t="inlineStr">
         <is>
-          <t>isoyear</t>
+          <t>isoweekday</t>
         </is>
       </c>
       <c r="B86" s="3" t="inlineStr">
@@ -2375,14 +2375,14 @@
       </c>
       <c r="D86" s="3" t="inlineStr">
         <is>
-          <t>Alias normalizado de iso_year.</t>
+          <t>Alias normalizado de iso_week_day.</t>
         </is>
       </c>
     </row>
     <row r="87" ht="42" customFormat="1" customHeight="1" s="1">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>now</t>
+          <t>iso_year</t>
         </is>
       </c>
       <c r="B87" s="3" t="inlineStr">
@@ -2397,14 +2397,14 @@
       </c>
       <c r="D87" s="3" t="inlineStr">
         <is>
-          <t>Asigna la fecha y hora local actual del sistema a la columna destino.</t>
+          <t>Extrae el año ISO 8601, que puede diferir del año calendario.</t>
         </is>
       </c>
     </row>
     <row r="88" ht="42" customFormat="1" customHeight="1" s="1">
       <c r="A88" s="3" t="inlineStr">
         <is>
-          <t>quarter</t>
+          <t>isoyear</t>
         </is>
       </c>
       <c r="B88" s="3" t="inlineStr">
@@ -2419,14 +2419,14 @@
       </c>
       <c r="D88" s="3" t="inlineStr">
         <is>
-          <t>Extrae el trimestre calendario como entero entre 1 y 4.</t>
+          <t>Alias normalizado de iso_year.</t>
         </is>
       </c>
     </row>
     <row r="89" ht="42" customFormat="1" customHeight="1" s="1">
       <c r="A89" s="3" t="inlineStr">
         <is>
-          <t>today</t>
+          <t>now</t>
         </is>
       </c>
       <c r="B89" s="3" t="inlineStr">
@@ -2441,14 +2441,14 @@
       </c>
       <c r="D89" s="3" t="inlineStr">
         <is>
-          <t>Asigna la fecha local actual del sistema sin hora a la columna destino.</t>
+          <t>Asigna la fecha y hora local actual del sistema a la columna destino.</t>
         </is>
       </c>
     </row>
     <row r="90" ht="42" customFormat="1" customHeight="1" s="1">
       <c r="A90" s="3" t="inlineStr">
         <is>
-          <t>week</t>
+          <t>quarter</t>
         </is>
       </c>
       <c r="B90" s="3" t="inlineStr">
@@ -2463,14 +2463,14 @@
       </c>
       <c r="D90" s="3" t="inlineStr">
         <is>
-          <t>Extrae el día de la semana como entero, lunes=0 hasta domingo=6.</t>
+          <t>Extrae el trimestre calendario como entero entre 1 y 4.</t>
         </is>
       </c>
     </row>
     <row r="91" ht="42" customFormat="1" customHeight="1" s="1">
       <c r="A91" s="3" t="inlineStr">
         <is>
-          <t>year</t>
+          <t>today</t>
         </is>
       </c>
       <c r="B91" s="3" t="inlineStr">
@@ -2485,14 +2485,14 @@
       </c>
       <c r="D91" s="3" t="inlineStr">
         <is>
-          <t>Extrae el año calendario como entero.</t>
+          <t>Asigna la fecha local actual del sistema sin hora a la columna destino.</t>
         </is>
       </c>
     </row>
     <row r="92" ht="42" customFormat="1" customHeight="1" s="1">
       <c r="A92" s="3" t="inlineStr">
         <is>
-          <t>dateadd</t>
+          <t>week</t>
         </is>
       </c>
       <c r="B92" s="3" t="inlineStr">
@@ -2502,19 +2502,19 @@
       </c>
       <c r="C92" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, unit: str | None = None, amount: int | None = None, create_new_column: bool = False, new_column_name: str | None = None, *, part: str | None = None, interval: int | None = None, replace: bool | None = None</t>
+          <t>df: pd.DataFrame, column: str, replace: bool = True, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D92" s="3" t="inlineStr">
         <is>
-          <t>Alias normalizado de date_add.</t>
+          <t>Extrae el día de la semana como entero, lunes=0 hasta domingo=6.</t>
         </is>
       </c>
     </row>
     <row r="93" ht="42" customFormat="1" customHeight="1" s="1">
       <c r="A93" s="3" t="inlineStr">
         <is>
-          <t>datediff</t>
+          <t>year</t>
         </is>
       </c>
       <c r="B93" s="3" t="inlineStr">
@@ -2524,19 +2524,19 @@
       </c>
       <c r="C93" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, start_column: str, end_column: str, unit: str = 'days', create_new_column: bool = False, new_column_name: str | None = None, *, part: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, replace: bool = True, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D93" s="3" t="inlineStr">
         <is>
-          <t>Alias normalizado de date_diff.</t>
+          <t>Extrae el año calendario como entero.</t>
         </is>
       </c>
     </row>
     <row r="94" ht="42" customFormat="1" customHeight="1" s="1">
       <c r="A94" s="3" t="inlineStr">
         <is>
-          <t>date_name</t>
+          <t>dateadd</t>
         </is>
       </c>
       <c r="B94" s="3" t="inlineStr">
@@ -2546,19 +2546,19 @@
       </c>
       <c r="C94" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, part: str, replace: bool = True, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, unit: str | None = None, amount: int | None = None, create_new_column: bool = False, new_column_name: str | None = None, *, part: str | None = None, interval: int | None = None, replace: bool | None = None</t>
         </is>
       </c>
       <c r="D94" s="3" t="inlineStr">
         <is>
-          <t>Devuelve el nombre en español del mes o del día de semana; año y trimestre se devuelven como texto.</t>
+          <t>Alias normalizado de date_add.</t>
         </is>
       </c>
     </row>
     <row r="95" ht="42" customFormat="1" customHeight="1" s="1">
       <c r="A95" s="3" t="inlineStr">
         <is>
-          <t>datename</t>
+          <t>datediff</t>
         </is>
       </c>
       <c r="B95" s="3" t="inlineStr">
@@ -2568,19 +2568,19 @@
       </c>
       <c r="C95" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, part: str, replace: bool = True, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, start_column: str, end_column: str, unit: str = 'days', create_new_column: bool = False, new_column_name: str | None = None, *, part: str | None = None</t>
         </is>
       </c>
       <c r="D95" s="3" t="inlineStr">
         <is>
-          <t>Alias normalizado de date_name.</t>
+          <t>Alias normalizado de date_diff.</t>
         </is>
       </c>
     </row>
     <row r="96" ht="42" customFormat="1" customHeight="1" s="1">
       <c r="A96" s="3" t="inlineStr">
         <is>
-          <t>month</t>
+          <t>date_name</t>
         </is>
       </c>
       <c r="B96" s="3" t="inlineStr">
@@ -2590,19 +2590,19 @@
       </c>
       <c r="C96" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, replace: bool = True, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, part: str, replace: bool = True, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D96" s="3" t="inlineStr">
         <is>
-          <t>Extrae el número del mes como entero entre 1 y 12.</t>
+          <t>Devuelve el nombre en español del mes o del día de semana; año y trimestre se devuelven como texto.</t>
         </is>
       </c>
     </row>
     <row r="97" ht="42" customFormat="1" customHeight="1" s="1">
       <c r="A97" s="3" t="inlineStr">
         <is>
-          <t>date add</t>
+          <t>datename</t>
         </is>
       </c>
       <c r="B97" s="3" t="inlineStr">
@@ -2612,19 +2612,19 @@
       </c>
       <c r="C97" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, unit: str | None = None, amount: int | None = None, create_new_column: bool = False, new_column_name: str | None = None, *, part: str | None = None, interval: int | None = None, replace: bool | None = None</t>
+          <t>df: pd.DataFrame, column: str, part: str, replace: bool = True, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D97" s="3" t="inlineStr">
         <is>
-          <t>Alias textual de date_add.</t>
+          <t>Alias normalizado de date_name.</t>
         </is>
       </c>
     </row>
     <row r="98" ht="42" customFormat="1" customHeight="1" s="1">
       <c r="A98" s="3" t="inlineStr">
         <is>
-          <t>date diff</t>
+          <t>month</t>
         </is>
       </c>
       <c r="B98" s="3" t="inlineStr">
@@ -2634,19 +2634,19 @@
       </c>
       <c r="C98" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, start_column: str, end_column: str, unit: str = 'days', create_new_column: bool = False, new_column_name: str | None = None, *, part: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, replace: bool = True, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D98" s="3" t="inlineStr">
         <is>
-          <t>Alias textual de date_diff.</t>
+          <t>Extrae el número del mes como entero entre 1 y 12.</t>
         </is>
       </c>
     </row>
     <row r="99" ht="42" customFormat="1" customHeight="1" s="1">
       <c r="A99" s="3" t="inlineStr">
         <is>
-          <t>date name</t>
+          <t>date add</t>
         </is>
       </c>
       <c r="B99" s="3" t="inlineStr">
@@ -2656,39 +2656,83 @@
       </c>
       <c r="C99" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, part: str, replace: bool = True, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, unit: str | None = None, amount: int | None = None, create_new_column: bool = False, new_column_name: str | None = None, *, part: str | None = None, interval: int | None = None, replace: bool | None = None</t>
         </is>
       </c>
       <c r="D99" s="3" t="inlineStr">
         <is>
-          <t>Alias textual de date_name.</t>
+          <t>Alias textual de date_add.</t>
         </is>
       </c>
     </row>
     <row r="100" ht="42" customHeight="1">
       <c r="A100" s="3" t="inlineStr">
         <is>
+          <t>date diff</t>
+        </is>
+      </c>
+      <c r="B100" s="3" t="inlineStr">
+        <is>
+          <t>DateTimeProcessor</t>
+        </is>
+      </c>
+      <c r="C100" s="3" t="inlineStr">
+        <is>
+          <t>df: pd.DataFrame, start_column: str, end_column: str, unit: str = 'days', create_new_column: bool = False, new_column_name: str | None = None, *, part: str | None = None</t>
+        </is>
+      </c>
+      <c r="D100" s="3" t="inlineStr">
+        <is>
+          <t>Alias textual de date_diff.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="3" t="inlineStr">
+        <is>
+          <t>date name</t>
+        </is>
+      </c>
+      <c r="B101" s="3" t="inlineStr">
+        <is>
+          <t>DateTimeProcessor</t>
+        </is>
+      </c>
+      <c r="C101" s="3" t="inlineStr">
+        <is>
+          <t>df: pd.DataFrame, column: str, part: str, replace: bool = True, new_column_name: str | None = None</t>
+        </is>
+      </c>
+      <c r="D101" s="3" t="inlineStr">
+        <is>
+          <t>Alias textual de date_name.</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="3" t="inlineStr">
+        <is>
           <t>concat_text</t>
         </is>
       </c>
-      <c r="B100" s="3" t="inlineStr">
+      <c r="B102" s="3" t="inlineStr">
         <is>
           <t>TextProcessor</t>
         </is>
       </c>
-      <c r="C100" s="3" t="inlineStr">
+      <c r="C102" s="3" t="inlineStr">
         <is>
           <t>df: pd.DataFrame, column_name: str, value: str, create_new_column: bool = False, new_column_name: str | None = None</t>
         </is>
       </c>
-      <c r="D100" s="3" t="inlineStr">
+      <c r="D102" s="3" t="inlineStr">
         <is>
           <t>Concatena un texto literal al contenido de la columna y reemplaza por defecto su valor; puede crear una columna nueva si se solicita.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D100"/>
+  <autoFilter ref="A1:D102"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>

<commit_message>
change replace or new_column parameters to create_new_column
</commit_message>
<xml_diff>
--- a/catalogo_operaciones.xlsx
+++ b/catalogo_operaciones.xlsx
@@ -610,7 +610,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, replace: bool = True, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, create_new_column: bool = False, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -632,7 +632,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, replace: bool = True, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, create_new_column: bool = False, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -654,7 +654,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, replace: bool = True, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, create_new_column: bool = False, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -676,7 +676,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, replace: bool = True, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, create_new_column: bool = False, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -698,7 +698,7 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, replace: bool = True, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, create_new_column: bool = False, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -720,7 +720,7 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column_day: str, column_month: str, column_year: str, replace: bool = False, new_column_name: str = 'date'</t>
+          <t>df: pd.DataFrame, column_day: str, column_month: str, column_year: str, create_new_column: bool = True, new_column_name: str = 'date'</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -808,12 +808,12 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, unit: str | None = None, amount: int | None = None, create_new_column: bool = False, new_column_name: str | None = None, *, part: str | None = None, interval: int | None = None, replace: bool | None = None</t>
+          <t>df: pd.DataFrame, column: str, unit: str | None = None, amount: int | None = None, create_new_column: bool = False, new_column_name: str | None = None, *, part: str | None = None, interval: int | None = None</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Agrega un intervalo entero de días, semanas, meses, trimestres, años, horas, minutos o segundos a una fecha. Acepta unit/amount o part/interval y reemplazo opcional.</t>
+          <t>Agrega un intervalo entero de días, semanas, meses, trimestres, años, horas, minutos o segundos a una fecha. Acepta unit/amount o part/interval y creación de columna opcional mediante create_new_column.</t>
         </is>
       </c>
     </row>
@@ -1094,7 +1094,7 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, new_column: bool = False, new_column_name: str | None = None, *, create_new_column: bool | None = None</t>
+          <t>df: pd.DataFrame, column: str, create_new_column: bool = False, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
@@ -1116,7 +1116,7 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, new_column: bool = False, new_column_name: str | None = None, *, create_new_column: bool | None = None</t>
+          <t>df: pd.DataFrame, column: str, create_new_column: bool = False, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
@@ -1160,7 +1160,7 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, new_column: bool = False, new_column_name: str | None = None, *, create_new_column: bool | None = None</t>
+          <t>df: pd.DataFrame, column: str, create_new_column: bool = False, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -1182,7 +1182,7 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, new_column: bool = False, new_column_name: str | None = None, *, create_new_column: bool | None = None</t>
+          <t>df: pd.DataFrame, column: str, create_new_column: bool = False, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -1204,7 +1204,7 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, new_column: bool = False, new_column_name: str | None = None, *, create_new_column: bool | None = None</t>
+          <t>df: pd.DataFrame, column: str, create_new_column: bool = False, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -1270,7 +1270,7 @@
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, value: float, new_column: bool = False, new_column_name: str | None = None, *, create_new_column: bool | None = None</t>
+          <t>df: pd.DataFrame, column: str, value: float, create_new_column: bool = False, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -1292,7 +1292,7 @@
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, decimals: int = 0, new_column: bool = False, new_column_name: str | None = None, *, create_new_column: bool | None = None</t>
+          <t>df: pd.DataFrame, column: str, decimals: int = 0, create_new_column: bool = False, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -1644,7 +1644,7 @@
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, new_type: str | None = None, *, target_type: str | None = None, create_new_column: bool | None = None, new_column: bool = False, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, new_type: str | None = None, *, target_type: str | None = None, create_new_column: bool = False, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
@@ -1666,7 +1666,7 @@
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, new_type: str | None = None, *, target_type: str | None = None, create_new_column: bool | None = None, new_column: bool = False, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, new_type: str | None = None, *, target_type: str | None = None, create_new_column: bool = False, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
@@ -1732,7 +1732,7 @@
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, new_column: bool = False, new_column_name: str | None = None, *, create_new_column: bool | None = None</t>
+          <t>df: pd.DataFrame, column: str, create_new_column: bool = False, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
@@ -1754,7 +1754,7 @@
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, new_column: bool = False, new_column_name: str | None = None, *, create_new_column: bool | None = None</t>
+          <t>df: pd.DataFrame, column: str, create_new_column: bool = False, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
@@ -1776,7 +1776,7 @@
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, new_column: bool = False, new_column_name: str | None = None, *, create_new_column: bool | None = None</t>
+          <t>df: pd.DataFrame, column: str, create_new_column: bool = False, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
@@ -1798,7 +1798,7 @@
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, new_column: bool = False, new_column_name: str | None = None, *, create_new_column: bool | None = None</t>
+          <t>df: pd.DataFrame, column: str, create_new_column: bool = False, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
@@ -2106,7 +2106,7 @@
       </c>
       <c r="C74" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, new_column: bool = False, new_column_name: str | None = None, *, create_new_column: bool | None = None</t>
+          <t>df: pd.DataFrame, column: str, create_new_column: bool = False, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D74" s="3" t="inlineStr">
@@ -2128,7 +2128,7 @@
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, new_column: bool = False, new_column_name: str | None = None, *, create_new_column: bool | None = None</t>
+          <t>df: pd.DataFrame, column: str, create_new_column: bool = False, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
@@ -2150,12 +2150,12 @@
       </c>
       <c r="C76" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, date_format: str, replace: bool = True, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, date_format: str, create_new_column: bool = False, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t>Convierte usando el formato indicado; los valores inválidos se convierten a NaT. Puede reemplazar o crear columna.</t>
+          <t>Convierte usando el formato indicado; los valores inválidos se convierten a NaT. Puede sobrescribir la columna fuente o crear una nueva con create_new_column.</t>
         </is>
       </c>
     </row>
@@ -2172,7 +2172,7 @@
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, date_format: str, replace: bool = True, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, date_format: str, create_new_column: bool = False, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D77" s="3" t="inlineStr">
@@ -2194,7 +2194,7 @@
       </c>
       <c r="C78" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, part: str, replace: bool = True, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, part: str, create_new_column: bool = False, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D78" s="3" t="inlineStr">
@@ -2216,7 +2216,7 @@
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, part: str, replace: bool = True, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, part: str, create_new_column: bool = False, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr">
@@ -2238,7 +2238,7 @@
       </c>
       <c r="C80" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, replace: bool = True, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, create_new_column: bool = False, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D80" s="3" t="inlineStr">
@@ -2260,7 +2260,7 @@
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, replace: bool = True, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, create_new_column: bool = False, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D81" s="3" t="inlineStr">
@@ -2282,7 +2282,7 @@
       </c>
       <c r="C82" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, replace: bool = True, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, create_new_column: bool = False, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D82" s="3" t="inlineStr">
@@ -2304,7 +2304,7 @@
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, replace: bool = True, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, create_new_column: bool = False, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D83" s="3" t="inlineStr">
@@ -2326,7 +2326,7 @@
       </c>
       <c r="C84" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, replace: bool = True, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, create_new_column: bool = False, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D84" s="3" t="inlineStr">
@@ -2348,7 +2348,7 @@
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, replace: bool = True, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, create_new_column: bool = False, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D85" s="3" t="inlineStr">
@@ -2370,7 +2370,7 @@
       </c>
       <c r="C86" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, replace: bool = True, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, create_new_column: bool = False, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D86" s="3" t="inlineStr">
@@ -2392,7 +2392,7 @@
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, replace: bool = True, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, create_new_column: bool = False, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D87" s="3" t="inlineStr">
@@ -2414,7 +2414,7 @@
       </c>
       <c r="C88" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, replace: bool = True, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, create_new_column: bool = False, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D88" s="3" t="inlineStr">
@@ -2436,7 +2436,7 @@
       </c>
       <c r="C89" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, replace: bool = True, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, create_new_column: bool = False, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D89" s="3" t="inlineStr">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="C90" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, replace: bool = True, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, create_new_column: bool = False, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D90" s="3" t="inlineStr">
@@ -2480,7 +2480,7 @@
       </c>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, replace: bool = True, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, create_new_column: bool = False, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D91" s="3" t="inlineStr">
@@ -2502,7 +2502,7 @@
       </c>
       <c r="C92" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, replace: bool = True, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, create_new_column: bool = False, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D92" s="3" t="inlineStr">
@@ -2524,7 +2524,7 @@
       </c>
       <c r="C93" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, replace: bool = True, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, create_new_column: bool = False, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D93" s="3" t="inlineStr">
@@ -2546,7 +2546,7 @@
       </c>
       <c r="C94" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, unit: str | None = None, amount: int | None = None, create_new_column: bool = False, new_column_name: str | None = None, *, part: str | None = None, interval: int | None = None, replace: bool | None = None</t>
+          <t>df: pd.DataFrame, column: str, unit: str | None = None, amount: int | None = None, create_new_column: bool = False, new_column_name: str | None = None, *, part: str | None = None, interval: int | None = None</t>
         </is>
       </c>
       <c r="D94" s="3" t="inlineStr">
@@ -2590,7 +2590,7 @@
       </c>
       <c r="C96" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, part: str, replace: bool = True, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, part: str, create_new_column: bool = False, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D96" s="3" t="inlineStr">
@@ -2612,7 +2612,7 @@
       </c>
       <c r="C97" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, part: str, replace: bool = True, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, part: str, create_new_column: bool = False, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D97" s="3" t="inlineStr">
@@ -2634,7 +2634,7 @@
       </c>
       <c r="C98" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, replace: bool = True, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, create_new_column: bool = False, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D98" s="3" t="inlineStr">
@@ -2656,7 +2656,7 @@
       </c>
       <c r="C99" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, unit: str | None = None, amount: int | None = None, create_new_column: bool = False, new_column_name: str | None = None, *, part: str | None = None, interval: int | None = None, replace: bool | None = None</t>
+          <t>df: pd.DataFrame, column: str, unit: str | None = None, amount: int | None = None, create_new_column: bool = False, new_column_name: str | None = None, *, part: str | None = None, interval: int | None = None</t>
         </is>
       </c>
       <c r="D99" s="3" t="inlineStr">
@@ -2700,7 +2700,7 @@
       </c>
       <c r="C101" s="3" t="inlineStr">
         <is>
-          <t>df: pd.DataFrame, column: str, part: str, replace: bool = True, new_column_name: str | None = None</t>
+          <t>df: pd.DataFrame, column: str, part: str, create_new_column: bool = False, new_column_name: str | None = None</t>
         </is>
       </c>
       <c r="D101" s="3" t="inlineStr">

</xml_diff>